<commit_message>
feat: implementar condicionales academicos (promedio < 10 e inasistencias > 4)
</commit_message>
<xml_diff>
--- a/Plantilla_Matricula_SICE.xlsx
+++ b/Plantilla_Matricula_SICE.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -435,11 +435,12 @@
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,25 +476,30 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Inasistencias</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Cédula Representante</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Nombre Representante</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Apellido Representante</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Teléfono Representante</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Correo Representante</t>
         </is>
@@ -530,27 +536,30 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>V-12345678</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Pedro</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Pérez</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>0412-1234567</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>pedro.perez@gmail.com</t>
         </is>
@@ -587,27 +596,30 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>V-13987654</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Carmen</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Rodríguez</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>0424-7654321</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>carmen.rod@gmail.com</t>
         </is>

</xml_diff>